<commit_message>
Add QA coverage for FEAT-DASH-07..15 and sync FR-DASH-02/04
Add FR-DASH-07 through 15 acceptance criteria (Given-When-Then + checklist,
matching the existing FR-DASH-01..06 style) and 43 new test cases
(TC-030..072) for the newer Dashboard analytics panels, with priority given
to the FR-DASH-11 DF/DHF conditional-display toggle. Update FR-DASH-02/04
wording to match the current stat tiles / weekly-chart implementation.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/03-testing/01-test-plan/v1/TEST-CASES.xlsx
+++ b/docs/03-testing/01-test-plan/v1/TEST-CASES.xlsx
@@ -892,7 +892,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J30"/>
+  <dimension ref="A1:J73"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -1866,6 +1866,2288 @@
         <v>17</v>
       </c>
     </row>
+    <row r="31" ht="60" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>TC-030</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>FR-DASH-02</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>Stat Tiles แสดงค่าจริงครบ 5 การ์ดหลังโหลดหน้า</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>ค่าเริ่มต้น</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. เปิดหน้า Dashboard
+2. รอโหลดเสร็จ
+3. ดู 5 การ์ด (รายใหม่วันนี้/รายใหม่นอกพื้นที่/ในพื้นที่สะสม/นอกพื้นที่สะสม/รวมผู้ป่วยสะสม)</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>ทั้ง 5 การ์ดแสดงตัวเลขจริง ไม่มีการ์ดใดค้าง "--"</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H31" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I31" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J31" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="60" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>TC-031</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>FR-DASH-02</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>ผลรวม "ในพื้นที่สะสม" + "นอกพื้นที่สะสม" = "รวมผู้ป่วยสะสม" พอดี</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>ค่าเริ่มต้น</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. บันทึกค่า 3 การ์ด
+2. เปลี่ยน filter โรคเป็น "ไข้เลือดออก"
+3. บันทึกค่าใหม่
+4. ทำซ้ำกับ filter เขตบริการเดี่ยว</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>ในพื้นที่สะสม + นอกพื้นที่สะสม = รวมผู้ป่วยสะสม พอดีทุกครั้ง (exact ไม่ใช่ประมาณ)</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I32" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J32" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="60" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>TC-032</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>FR-DASH-02</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>พื้นหลัง Stat Tile ใช้โทนดินอ่อนแยกหมวด ไม่ใช่สีสถานะ</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>ค่าเริ่มต้น</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>1. ตรวจสอบ class พื้นหลังของ 5 การ์ด</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>ไม่มีการ์ดใดใช้สีเขียว/เหลือง/แดงแบบ risk level ของ Zone Risk Grid</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H33" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I33" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J33" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="60" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>TC-033</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>FR-DASH-02</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>Stat Tiles อัปเดตตาม filter</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>ค่าเริ่มต้น</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. เปลี่ยน filter โรค+เขตบริการ+ช่วงวันที่พร้อมกัน
+2. สังเกตค่า 5 การ์ด</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>ค่าทั้ง 5 การ์ดเปลี่ยนตรงกับ filter ใหม่ทันที ไม่ค้างค่าเดิม</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H34" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I34" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J34" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="60" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>TC-034</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>FR-DASH-04</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>กราฟรายสัปดาห์แสดง 52 สัปดาห์เสมอ ไม่ผูกกับ filter ช่วงวันที่</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>ค่าเริ่มต้น</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. บันทึกจำนวนจุดข้อมูล/รูปกราฟรายสัปดาห์
+2. เปลี่ยน filter ช่วงวันที่เป็น 7 วัน แล้ว 30 วัน
+3. เทียบกราฟรายสัปดาห์ทั้ง 2 ครั้ง</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>กราฟรายสัปดาห์แสดง 52 สัปดาห์เท่าเดิมทุกครั้ง ไม่เปลี่ยนตามตัวกรองช่วงวันที่</t>
+        </is>
+      </c>
+      <c r="G35" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H35" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I35" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J35" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="60" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>TC-035</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>FR-DASH-04</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>Legend กราฟรายสัปดาห์แสดงปีถูกต้อง</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>ค่าเริ่มต้น</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>1. ดู legend กราฟรายสัปดาห์</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>แสดง "ปีปัจจุบัน" และ "ค่ามัธยฐานปีก่อน" พร้อมปี พ.ศ. ถูกต้อง</t>
+        </is>
+      </c>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H36" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I36" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J36" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="60" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>TC-036</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>FR-DASH-04</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>Subtitle กราฟรายวัน/รายสัปดาห์แยกแยะกันชัดเจนและอัปเดตตาม filter</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>ค่าเริ่มต้น</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. เปลี่ยน filter โรคเป็น "ไข้หวัดใหญ่" และเขตบริการเป็น "เขตบริการ 2"
+2. อ่าน subtitle ทั้ง 2 กราฟ</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>Subtitle ทั้งคู่ระบุโรค/เขตบริการตรงกับ filter ปัจจุบัน ไม่มีข้อความสลับกัน</t>
+        </is>
+      </c>
+      <c r="G37" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H37" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I37" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J37" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="60" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>TC-037</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>FR-DASH-04</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>กราฟทั้ง 2 เรนเดอร์ปกติเมื่อ filter มีเคสน้อยมาก</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>ค่าเริ่มต้น</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. เลือกโรค "อาหารเป็นพิษ" + เขตบริการ 1
+2. ดูกราฟรายวันและรายสัปดาห์</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>ทั้ง 2 กราฟเรนเดอร์ได้ปกติ ไม่มี error/แท่ง-เส้นหายไปทั้งหมด</t>
+        </is>
+      </c>
+      <c r="G38" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H38" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I38" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J38" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="60" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>TC-038</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>FR-DASH-07</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>อัตราป่วยต่อแสนประชากร คำนวณถูกต้อง (happy path)</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>ค่าเริ่มต้น</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. บันทึกค่าเคสสะสมรวมและประชากรรวม 4 เขต
+2. เทียบกับค่าการ์ดอัตราป่วย</t>
+        </is>
+      </c>
+      <c r="F39" s="2" t="inlineStr">
+        <is>
+          <t>ค่าการ์ด = (เคสสะสม ÷ ประชากรรวม) × 100,000 ตรงกับสูตร</t>
+        </is>
+      </c>
+      <c r="G39" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H39" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I39" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J39" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="60" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>TC-039</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>FR-DASH-07</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>เลือกเขตบริการเดียว ตัวหารเปลี่ยนเป็นประชากรเขตนั้น</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>ค่าเริ่มต้น</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. เลือก filter เขตบริการ = "เขตบริการ 2"
+2. เทียบค่าการ์ดกับสูตรที่ใช้ประชากรเขต 2 เท่านั้น</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="inlineStr">
+        <is>
+          <t>ค่าการ์ดตรงกับสูตร ไม่ใช่ประชากรรวม 4 เขต</t>
+        </is>
+      </c>
+      <c r="G40" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H40" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I40" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J40" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="60" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>TC-040</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>FR-DASH-07</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>เปลี่ยนช่วงวันที่ ตัวเศษ (เคสสะสม) เปลี่ยนตาม</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>ค่าเริ่มต้น</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. บันทึกค่าการ์ดที่ 14 วัน
+2. เปลี่ยนเป็น 30 วัน
+3. เทียบค่าการ์ดใหม่</t>
+        </is>
+      </c>
+      <c r="F41" s="2" t="inlineStr">
+        <is>
+          <t>ค่าการ์ดเปลี่ยนตามจำนวนเคสสะสมของช่วง 30 วัน สูตรยังถูกต้อง</t>
+        </is>
+      </c>
+      <c r="G41" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H41" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I41" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J41" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="60" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>TC-041</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>FR-DASH-07</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>(Edge) filter ที่ไม่มีเคสตรงเงื่อนไข อัตราป่วยแสดง 0 ไม่ error</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>ค่าเริ่มต้น</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>1. เลือกโรค+เขตบริการที่ไม่มีเคสในช่วง 7 วัน</t>
+        </is>
+      </c>
+      <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t>การ์ดแสดง 0.0 หรือค่าต่ำสุดที่ถูกต้อง ไม่แสดง NaN/error/ค้าง "--"</t>
+        </is>
+      </c>
+      <c r="G42" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H42" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I42" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J42" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="60" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>TC-042</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>FR-DASH-08</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>ตารางเพศแสดง 2 แถวถูกต้อง (happy path)</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>ค่าเริ่มต้น</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. ดูตารางเพศ
+2. บันทึกจำนวนเคสชาย+หญิง</t>
+        </is>
+      </c>
+      <c r="F43" s="2" t="inlineStr">
+        <is>
+          <t>มี 2 แถว จำนวนรวมกันเท่ากับเคสสะสมรวมของ filter ปัจจุบันพอดี</t>
+        </is>
+      </c>
+      <c r="G43" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H43" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I43" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J43" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="60" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>TC-043</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>FR-DASH-08</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>ร้อยละชาย+หญิง รวมกัน ≈100%</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>ค่าเริ่มต้น</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. อ่านร้อยละ 2 แถว
+2. บวกกัน</t>
+        </is>
+      </c>
+      <c r="F44" s="2" t="inlineStr">
+        <is>
+          <t>ผลรวม ≈100% (คลาดเคลื่อนไม่เกิน ±0.2%)</t>
+        </is>
+      </c>
+      <c r="G44" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H44" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I44" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J44" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="60" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>TC-044</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>FR-DASH-08</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>Progress bar ยาวตามสัดส่วนร้อยละ</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>ค่าเริ่มต้น</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
+          <t>1. ตรวจสอบ width ของ progress bar แต่ละแถว เทียบกับร้อยละที่แสดง</t>
+        </is>
+      </c>
+      <c r="F45" s="2" t="inlineStr">
+        <is>
+          <t>ความยาว bar เป็นสัดส่วนตรงกับร้อยละของแถวนั้น</t>
+        </is>
+      </c>
+      <c r="G45" s="2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H45" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I45" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J45" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="60" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>TC-045</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>FR-DASH-08</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>ตารางเพศอัปเดตตาม filter</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>ค่าเริ่มต้น</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. เปลี่ยน filter โรคเป็น "โควิด-19"
+2. ดูตารางเพศใหม่</t>
+        </is>
+      </c>
+      <c r="F46" s="2" t="inlineStr">
+        <is>
+          <t>จำนวนเคส/ร้อยละ/progress bar ทั้ง 2 แถวเปลี่ยนให้ตรงกับข้อมูลโควิด-19</t>
+        </is>
+      </c>
+      <c r="G46" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H46" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I46" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J46" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="60" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>TC-046</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>FR-DASH-09</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="inlineStr">
+        <is>
+          <t>ตารางกลุ่มอายุแสดงครบ 5 ช่วงตามลำดับ</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>ค่าเริ่มต้น</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="inlineStr">
+        <is>
+          <t>1. ดูตารางกลุ่มอายุ</t>
+        </is>
+      </c>
+      <c r="F47" s="2" t="inlineStr">
+        <is>
+          <t>แสดง 5 แถวเรียงลำดับ 05-14, 15-24, 25-34, 35-44, 45-54 ไม่ขาด/สลับ</t>
+        </is>
+      </c>
+      <c r="G47" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H47" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I47" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J47" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="60" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>TC-047</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>FR-DASH-09</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>ร้อยละของ 5 ช่วงอายุรวมกัน ≈100%</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>ค่าเริ่มต้น</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. อ่านร้อยละทั้ง 5 แถว
+2. บวกกัน</t>
+        </is>
+      </c>
+      <c r="F48" s="2" t="inlineStr">
+        <is>
+          <t>ผลรวม ≈100%</t>
+        </is>
+      </c>
+      <c r="G48" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H48" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I48" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J48" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="60" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>TC-048</t>
+        </is>
+      </c>
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>FR-DASH-09</t>
+        </is>
+      </c>
+      <c r="C49" s="2" t="inlineStr">
+        <is>
+          <t>อัตราป่วยต่อแสนปกครองต่อช่วงอายุ คำนวณแยกจากร้อยละเคส</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="inlineStr">
+        <is>
+          <t>ค่าเริ่มต้น</t>
+        </is>
+      </c>
+      <c r="E49" s="2" t="inlineStr">
+        <is>
+          <t>1. เทียบคอลัมน์อัตราป่วยกับคอลัมน์ร้อยละของแต่ละแถว</t>
+        </is>
+      </c>
+      <c r="F49" s="2" t="inlineStr">
+        <is>
+          <t>ค่าทั้ง 2 คอลัมน์คำนวณจากสูตรคนละสูตร ไม่จำเป็นต้องมีสัดส่วนเดียวกัน</t>
+        </is>
+      </c>
+      <c r="G49" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H49" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I49" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J49" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="60" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>TC-049</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>FR-DASH-09</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>ตารางกลุ่มอายุอัปเดตตาม filter</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>ค่าเริ่มต้น</t>
+        </is>
+      </c>
+      <c r="E50" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. เปลี่ยน filter ช่วงวันที่เป็น 30 วัน
+2. ดูตารางใหม่</t>
+        </is>
+      </c>
+      <c r="F50" s="2" t="inlineStr">
+        <is>
+          <t>จำนวนเคส/ร้อยละ/อัตราป่วยทั้ง 5 แถวอัปเดตตรงกับ filter ใหม่</t>
+        </is>
+      </c>
+      <c r="G50" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H50" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I50" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J50" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="60" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>TC-050</t>
+        </is>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>FR-DASH-10</t>
+        </is>
+      </c>
+      <c r="C51" s="2" t="inlineStr">
+        <is>
+          <t>การ์ดอายุมากที่สุด/มัธยฐาน/น้อยที่สุด ตรงกับข้อมูลตาราง FR-DASH-09</t>
+        </is>
+      </c>
+      <c r="D51" s="2" t="inlineStr">
+        <is>
+          <t>ค่าเริ่มต้น</t>
+        </is>
+      </c>
+      <c r="E51" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. ดูค่า 3 การ์ด
+2. เทียบกับช่วงอายุที่มีเคสในตาราง FR-DASH-09</t>
+        </is>
+      </c>
+      <c r="F51" s="2" t="inlineStr">
+        <is>
+          <t>อายุมากที่สุด/น้อยที่สุดอยู่ในช่วงอายุที่มีเคส ค่ามัธยฐานอยู่ระหว่างค่าทั้งสอง</t>
+        </is>
+      </c>
+      <c r="G51" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H51" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I51" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J51" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="60" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>TC-051</t>
+        </is>
+      </c>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>FR-DASH-10</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t>มัธยฐานคำนวณถูกต้องกรณีจำนวนเคสเป็นเลขคี่</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t>ค่าเริ่มต้น</t>
+        </is>
+      </c>
+      <c r="E52" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. เลือก filter ที่ได้จำนวนเคสรวมเป็นเลขคี่
+2. ตรวจสอบค่ามัธยฐาน</t>
+        </is>
+      </c>
+      <c r="F52" s="2" t="inlineStr">
+        <is>
+          <t>ค่ามัธยฐาน = ค่ากลางจริงของอายุที่เรียงแล้ว</t>
+        </is>
+      </c>
+      <c r="G52" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H52" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I52" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J52" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="60" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>TC-052</t>
+        </is>
+      </c>
+      <c r="B53" s="2" t="inlineStr">
+        <is>
+          <t>FR-DASH-10</t>
+        </is>
+      </c>
+      <c r="C53" s="2" t="inlineStr">
+        <is>
+          <t>(Edge) มัธยฐานคำนวณถูกต้องกรณีจำนวนเคสเป็นเลขคู่</t>
+        </is>
+      </c>
+      <c r="D53" s="2" t="inlineStr">
+        <is>
+          <t>ค่าเริ่มต้น</t>
+        </is>
+      </c>
+      <c r="E53" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. เลือก filter ที่ได้จำนวนเคสรวมเป็นเลขคู่
+2. ตรวจสอบค่ามัธยฐาน</t>
+        </is>
+      </c>
+      <c r="F53" s="2" t="inlineStr">
+        <is>
+          <t>ค่ามัธยฐาน = ค่าเฉลี่ยของ 2 ค่ากลาง (ปัดเป็นจำนวนเต็ม)</t>
+        </is>
+      </c>
+      <c r="G53" s="2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H53" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I53" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J53" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="60" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>TC-053</t>
+        </is>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>FR-DASH-10</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t>(Edge) ไม่มีเคสตรง filter การ์ดแสดง "-"</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t>ค่าเริ่มต้น</t>
+        </is>
+      </c>
+      <c r="E54" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. เลือก filter ที่ไม่มีเคสตรงเงื่อนไขเลย
+2. ดู 3 การ์ด</t>
+        </is>
+      </c>
+      <c r="F54" s="2" t="inlineStr">
+        <is>
+          <t>ทั้ง 3 การ์ดแสดง "-" ไม่ error ไม่ค้างค่าเดิม</t>
+        </is>
+      </c>
+      <c r="G54" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H54" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I54" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J54" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="60" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>TC-054</t>
+        </is>
+      </c>
+      <c r="B55" s="2" t="inlineStr">
+        <is>
+          <t>FR-DASH-11</t>
+        </is>
+      </c>
+      <c r="C55" s="2" t="inlineStr">
+        <is>
+          <t>[Toggle ทางที่ 1] เลือกโรค = ไข้เลือดออก panel DF/DHF แสดง</t>
+        </is>
+      </c>
+      <c r="D55" s="2" t="inlineStr">
+        <is>
+          <t>ค่าเริ่มต้น</t>
+        </is>
+      </c>
+      <c r="E55" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. เปิด filter โรค
+2. เลือก "ไข้เลือดออก (Dengue Fever)"
+3. ดู panel donut chart DF/DHF</t>
+        </is>
+      </c>
+      <c r="F55" s="2" t="inlineStr">
+        <is>
+          <t>Panel แสดง donut chart + legend สัดส่วน DF/DHF ผลรวม DF+DHF = เคสไข้เลือดออกทั้งหมดตาม filter note ต้องซ่อน</t>
+        </is>
+      </c>
+      <c r="G55" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H55" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I55" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J55" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="60" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>TC-055</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t>FR-DASH-11</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
+          <t>[Toggle ทางที่ 2] เลือกโรค = ทุกโรค panel DF/DHF ซ่อน+มี note</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="inlineStr">
+        <is>
+          <t>ต่อจากสถานะเลือกไข้เลือดออกไว้</t>
+        </is>
+      </c>
+      <c r="E56" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. เปลี่ยน filter โรคเป็น "ทุกโรค (All Diseases)"
+2. ดู panel</t>
+        </is>
+      </c>
+      <c r="F56" s="2" t="inlineStr">
+        <is>
+          <t>Donut chart + legend ซ่อน แสดง note "แสดงเมื่อเลือกตัวกรองโรคเป็นไข้เลือดออก (Dengue Fever) เท่านั้น"</t>
+        </is>
+      </c>
+      <c r="G56" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H56" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I56" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J56" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="60" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A57" s="2" t="inlineStr">
+        <is>
+          <t>TC-056</t>
+        </is>
+      </c>
+      <c r="B57" s="2" t="inlineStr">
+        <is>
+          <t>FR-DASH-11</t>
+        </is>
+      </c>
+      <c r="C57" s="2" t="inlineStr">
+        <is>
+          <t>[Toggle ทางที่ 2 เพิ่ม] เลือกโรคอื่นที่ไม่ใช่ไข้เลือดออก panel ซ่อน+มี note</t>
+        </is>
+      </c>
+      <c r="D57" s="2" t="inlineStr">
+        <is>
+          <t>ค่าเริ่มต้น</t>
+        </is>
+      </c>
+      <c r="E57" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. เลือก filter โรคเป็น "ไข้หวัดใหญ่"
+2. ดู panel
+3. ทำซ้ำกับ "โควิด-19", "มือ เท้า ปาก", "อาหารเป็นพิษ"</t>
+        </is>
+      </c>
+      <c r="F57" s="2" t="inlineStr">
+        <is>
+          <t>Panel ซ่อนและแสดง note เดียวกันในทุกกรณีที่ไม่ใช่ไข้เลือดออก</t>
+        </is>
+      </c>
+      <c r="G57" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H57" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I57" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J57" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="60" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>TC-057</t>
+        </is>
+      </c>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>FR-DASH-11</t>
+        </is>
+      </c>
+      <c r="C58" s="2" t="inlineStr">
+        <is>
+          <t>สลับกลับไปเลือกไข้เลือดออกอีกครั้ง panel ต้องกลับมาแสดงถูกต้อง (regression toggle)</t>
+        </is>
+      </c>
+      <c r="D58" s="2" t="inlineStr">
+        <is>
+          <t>ต่อจากสถานะ filter โรคอื่น</t>
+        </is>
+      </c>
+      <c r="E58" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. เปลี่ยน filter โรคกลับเป็น "ไข้เลือดออก (Dengue Fever)"
+2. ดู panel</t>
+        </is>
+      </c>
+      <c r="F58" s="2" t="inlineStr">
+        <is>
+          <t>Panel donut chart + legend กลับมาแสดงพร้อมข้อมูลที่ตรงกับ filter ปัจจุบัน ไม่ค้างสถานะซ่อน</t>
+        </is>
+      </c>
+      <c r="G58" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H58" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I58" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J58" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="60" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A59" s="2" t="inlineStr">
+        <is>
+          <t>TC-058</t>
+        </is>
+      </c>
+      <c r="B59" s="2" t="inlineStr">
+        <is>
+          <t>FR-DASH-12</t>
+        </is>
+      </c>
+      <c r="C59" s="2" t="inlineStr">
+        <is>
+          <t>ตารางอาชีพแสดงครบ 5 หมวด ผลรวมเคสตรงกับเคสสะสม</t>
+        </is>
+      </c>
+      <c r="D59" s="2" t="inlineStr">
+        <is>
+          <t>ค่าเริ่มต้น</t>
+        </is>
+      </c>
+      <c r="E59" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. ดูตารางอาชีพ
+2. รวมจำนวนเคสทั้ง 5 หมวด</t>
+        </is>
+      </c>
+      <c r="F59" s="2" t="inlineStr">
+        <is>
+          <t>มีครบ 5 หมวด ผลรวม = เคสสะสมรวมของ filter ปัจจุบันพอดี</t>
+        </is>
+      </c>
+      <c r="G59" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H59" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I59" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J59" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="60" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t>TC-059</t>
+        </is>
+      </c>
+      <c r="B60" s="2" t="inlineStr">
+        <is>
+          <t>FR-DASH-12</t>
+        </is>
+      </c>
+      <c r="C60" s="2" t="inlineStr">
+        <is>
+          <t>ร้อยละ 5 หมวดอาชีพรวมกัน ≈100%</t>
+        </is>
+      </c>
+      <c r="D60" s="2" t="inlineStr">
+        <is>
+          <t>ค่าเริ่มต้น</t>
+        </is>
+      </c>
+      <c r="E60" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. อ่านร้อยละ 5 หมวด
+2. บวกกัน</t>
+        </is>
+      </c>
+      <c r="F60" s="2" t="inlineStr">
+        <is>
+          <t>ผลรวม ≈100%</t>
+        </is>
+      </c>
+      <c r="G60" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H60" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I60" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J60" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="60" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A61" s="2" t="inlineStr">
+        <is>
+          <t>TC-060</t>
+        </is>
+      </c>
+      <c r="B61" s="2" t="inlineStr">
+        <is>
+          <t>FR-DASH-12</t>
+        </is>
+      </c>
+      <c r="C61" s="2" t="inlineStr">
+        <is>
+          <t>ตารางอาชีพอัปเดตตาม filter</t>
+        </is>
+      </c>
+      <c r="D61" s="2" t="inlineStr">
+        <is>
+          <t>ค่าเริ่มต้น</t>
+        </is>
+      </c>
+      <c r="E61" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. เปลี่ยน filter เขตบริการเป็นเขตเดียว
+2. ดูตารางใหม่</t>
+        </is>
+      </c>
+      <c r="F61" s="2" t="inlineStr">
+        <is>
+          <t>จำนวนเคส/ร้อยละของ 5 หมวดอัปเดตตรงกับข้อมูลที่กรอง</t>
+        </is>
+      </c>
+      <c r="G61" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H61" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I61" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J61" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="60" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A62" s="2" t="inlineStr">
+        <is>
+          <t>TC-061</t>
+        </is>
+      </c>
+      <c r="B62" s="2" t="inlineStr">
+        <is>
+          <t>FR-DASH-13</t>
+        </is>
+      </c>
+      <c r="C62" s="2" t="inlineStr">
+        <is>
+          <t>ตาราง Top 8 ชุมชนเรียงจากมากไปน้อยถูกต้อง</t>
+        </is>
+      </c>
+      <c r="D62" s="2" t="inlineStr">
+        <is>
+          <t>ค่าเริ่มต้น</t>
+        </is>
+      </c>
+      <c r="E62" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. ดูตารางชุมชน
+2. ตรวจสอบลำดับจำนวนเคสของแต่ละแถว</t>
+        </is>
+      </c>
+      <c r="F62" s="2" t="inlineStr">
+        <is>
+          <t>แสดงไม่เกิน 8 แถว เรียงจำนวนเคสมากไปน้อยถูกต้อง</t>
+        </is>
+      </c>
+      <c r="G62" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H62" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I62" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J62" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="63" ht="60" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A63" s="2" t="inlineStr">
+        <is>
+          <t>TC-062</t>
+        </is>
+      </c>
+      <c r="B63" s="2" t="inlineStr">
+        <is>
+          <t>FR-DASH-13</t>
+        </is>
+      </c>
+      <c r="C63" s="2" t="inlineStr">
+        <is>
+          <t>Badge เขตบริการ/ทีมสอบสวนโรคต่อชุมชนถูกต้อง</t>
+        </is>
+      </c>
+      <c r="D63" s="2" t="inlineStr">
+        <is>
+          <t>ค่าเริ่มต้น</t>
+        </is>
+      </c>
+      <c r="E63" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. เลือกชุมชนแถวใดแถวหนึ่ง
+2. เทียบชื่อเขตบริการ/badge ทีมกับข้อมูลใน Zone Risk Grid</t>
+        </is>
+      </c>
+      <c r="F63" s="2" t="inlineStr">
+        <is>
+          <t>เขตบริการ/ทีมสอบสวนโรคตรงกับที่ Zone Risk Grid แสดงสำหรับชุมชนนั้น</t>
+        </is>
+      </c>
+      <c r="G63" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H63" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I63" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J63" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="64" ht="60" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A64" s="2" t="inlineStr">
+        <is>
+          <t>TC-063</t>
+        </is>
+      </c>
+      <c r="B64" s="2" t="inlineStr">
+        <is>
+          <t>FR-DASH-13</t>
+        </is>
+      </c>
+      <c r="C64" s="2" t="inlineStr">
+        <is>
+          <t>(Edge) ผลรวมเคสของชุมชน Top 8 ไม่เกินยอดรวมระดับเขตบริการ</t>
+        </is>
+      </c>
+      <c r="D64" s="2" t="inlineStr">
+        <is>
+          <t>เลือก filter เขตบริการ = เขตเดียว</t>
+        </is>
+      </c>
+      <c r="E64" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. รวมจำนวนเคสของทุกแถวในตารางชุมชน
+2. เทียบกับจำนวนเคสสะสมของเขตบริการนั้นใน Zone Risk Grid</t>
+        </is>
+      </c>
+      <c r="F64" s="2" t="inlineStr">
+        <is>
+          <t>ผลรวมเคสของชุมชนที่แสดง ≤ จำนวนเคสสะสมของเขตบริการนั้น</t>
+        </is>
+      </c>
+      <c r="G64" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H64" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I64" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J64" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="65" ht="60" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A65" s="2" t="inlineStr">
+        <is>
+          <t>TC-064</t>
+        </is>
+      </c>
+      <c r="B65" s="2" t="inlineStr">
+        <is>
+          <t>FR-DASH-13</t>
+        </is>
+      </c>
+      <c r="C65" s="2" t="inlineStr">
+        <is>
+          <t>(Edge) Empty state เมื่อไม่มีชุมชนตรง filter</t>
+        </is>
+      </c>
+      <c r="D65" s="2" t="inlineStr">
+        <is>
+          <t>ค่าเริ่มต้น</t>
+        </is>
+      </c>
+      <c r="E65" s="2" t="inlineStr">
+        <is>
+          <t>1. เลือก filter ที่ไม่มีเคสตรงเงื่อนไขเลย</t>
+        </is>
+      </c>
+      <c r="F65" s="2" t="inlineStr">
+        <is>
+          <t>ตารางแสดงข้อความ empty state แทนแถวว่างเปล่า</t>
+        </is>
+      </c>
+      <c r="G65" s="2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H65" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I65" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J65" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="66" ht="60" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A66" s="2" t="inlineStr">
+        <is>
+          <t>TC-065</t>
+        </is>
+      </c>
+      <c r="B66" s="2" t="inlineStr">
+        <is>
+          <t>FR-DASH-13</t>
+        </is>
+      </c>
+      <c r="C66" s="2" t="inlineStr">
+        <is>
+          <t>Top 8 คำนวณใหม่เมื่อเปลี่ยน filter</t>
+        </is>
+      </c>
+      <c r="D66" s="2" t="inlineStr">
+        <is>
+          <t>ค่าเริ่มต้น</t>
+        </is>
+      </c>
+      <c r="E66" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. บันทึกรายชื่อ Top 8 เดิม
+2. เปลี่ยน filter โรค
+3. เทียบรายชื่อ/ลำดับใหม่</t>
+        </is>
+      </c>
+      <c r="F66" s="2" t="inlineStr">
+        <is>
+          <t>รายชื่อและลำดับ Top 8 เปลี่ยนให้ตรงกับข้อมูลที่กรองใหม่</t>
+        </is>
+      </c>
+      <c r="G66" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H66" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I66" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J66" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="67" ht="60" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A67" s="2" t="inlineStr">
+        <is>
+          <t>TC-066</t>
+        </is>
+      </c>
+      <c r="B67" s="2" t="inlineStr">
+        <is>
+          <t>FR-DASH-14</t>
+        </is>
+      </c>
+      <c r="C67" s="2" t="inlineStr">
+        <is>
+          <t>ตารางเขตบริการแสดงครบ 4 เขต เรียงตามอัตราป่วยสูงไปต่ำ (happy path)</t>
+        </is>
+      </c>
+      <c r="D67" s="2" t="inlineStr">
+        <is>
+          <t>ค่าเริ่มต้น (เขตบริการ = ทุกเขตบริการ)</t>
+        </is>
+      </c>
+      <c r="E67" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. ดูตารางเขตบริการ
+2. ตรวจสอบลำดับคอลัมน์อัตราป่วย</t>
+        </is>
+      </c>
+      <c r="F67" s="2" t="inlineStr">
+        <is>
+          <t>แสดงครบ 4 เขต เรียงจากอัตราป่วยสูงไปต่ำถูกต้อง</t>
+        </is>
+      </c>
+      <c r="G67" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H67" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I67" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J67" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="68" ht="60" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A68" s="2" t="inlineStr">
+        <is>
+          <t>TC-067</t>
+        </is>
+      </c>
+      <c r="B68" s="2" t="inlineStr">
+        <is>
+          <t>FR-DASH-14</t>
+        </is>
+      </c>
+      <c r="C68" s="2" t="inlineStr">
+        <is>
+          <t>เปลี่ยน filter โรค ตารางคำนวณและเรียงลำดับใหม่</t>
+        </is>
+      </c>
+      <c r="D68" s="2" t="inlineStr">
+        <is>
+          <t>ค่าเริ่มต้น</t>
+        </is>
+      </c>
+      <c r="E68" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. บันทึกลำดับเขตเดิม
+2. เปลี่ยน filter โรคเป็น "โควิด-19"
+3. เทียบลำดับใหม่</t>
+        </is>
+      </c>
+      <c r="F68" s="2" t="inlineStr">
+        <is>
+          <t>อัตราป่วยเปลี่ยน และลำดับแถว re-sort ใหม่ถูกต้อง</t>
+        </is>
+      </c>
+      <c r="G68" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H68" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I68" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J68" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="69" ht="60" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A69" s="2" t="inlineStr">
+        <is>
+          <t>TC-068</t>
+        </is>
+      </c>
+      <c r="B69" s="2" t="inlineStr">
+        <is>
+          <t>FR-DASH-14</t>
+        </is>
+      </c>
+      <c r="C69" s="2" t="inlineStr">
+        <is>
+          <t>เลือก filter เขตบริการเดียว ตารางแสดงเฉพาะเขตนั้น (filter ไม่ dim)</t>
+        </is>
+      </c>
+      <c r="D69" s="2" t="inlineStr">
+        <is>
+          <t>ค่าเริ่มต้น</t>
+        </is>
+      </c>
+      <c r="E69" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. เลือก filter เขตบริการ = "เขตบริการ 3"
+2. ดูตารางเขตบริการ</t>
+        </is>
+      </c>
+      <c r="F69" s="2" t="inlineStr">
+        <is>
+          <t>ตารางแสดงเฉพาะแถว "เขตบริการ 3" เขตเดียว (ไม่แสดง 4 แถวแบบ dim เหมือน Zone Risk Grid)</t>
+        </is>
+      </c>
+      <c r="G69" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H69" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I69" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J69" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="70" ht="60" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A70" s="2" t="inlineStr">
+        <is>
+          <t>TC-069</t>
+        </is>
+      </c>
+      <c r="B70" s="2" t="inlineStr">
+        <is>
+          <t>FR-DASH-14</t>
+        </is>
+      </c>
+      <c r="C70" s="2" t="inlineStr">
+        <is>
+          <t>(Regression) ลำดับถูกต้องข้าม filter หลายชุด</t>
+        </is>
+      </c>
+      <c r="D70" s="2" t="inlineStr">
+        <is>
+          <t>ค่าเริ่มต้น</t>
+        </is>
+      </c>
+      <c r="E70" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. ทดสอบ filter ชุดที่ 1 บันทึกลำดับ
+2. ทดสอบ filter ชุดที่ 2 บันทึกลำดับ
+3. เทียบว่าลำดับสอดคล้องกับอัตราป่วยจริง</t>
+        </is>
+      </c>
+      <c r="F70" s="2" t="inlineStr">
+        <is>
+          <t>ลำดับเขตบริการเรียงจากอัตราป่วยสูงไปต่ำถูกต้องในทุกชุด filter</t>
+        </is>
+      </c>
+      <c r="G70" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H70" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I70" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J70" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="71" ht="60" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A71" s="2" t="inlineStr">
+        <is>
+          <t>TC-070</t>
+        </is>
+      </c>
+      <c r="B71" s="2" t="inlineStr">
+        <is>
+          <t>FR-DASH-15</t>
+        </is>
+      </c>
+      <c r="C71" s="2" t="inlineStr">
+        <is>
+          <t>ตารางป่วยจาก 2 แถว ค่าตรงกับ Stat Tiles (happy path)</t>
+        </is>
+      </c>
+      <c r="D71" s="2" t="inlineStr">
+        <is>
+          <t>ค่าเริ่มต้น</t>
+        </is>
+      </c>
+      <c r="E71" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. บันทึกค่า "นอกพื้นที่สะสม" และ "รายใหม่วันนี้" จาก Stat Tiles
+2. ดูตารางป่วยจาก</t>
+        </is>
+      </c>
+      <c r="F71" s="2" t="inlineStr">
+        <is>
+          <t>แถว "เริ่มป่วยจากนอกพื้นที่ (สะสม)" = ค่า "นอกพื้นที่สะสม" ใน Stat Tiles พอดี</t>
+        </is>
+      </c>
+      <c r="G71" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H71" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I71" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J71" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="72" ht="60" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A72" s="2" t="inlineStr">
+        <is>
+          <t>TC-071</t>
+        </is>
+      </c>
+      <c r="B72" s="2" t="inlineStr">
+        <is>
+          <t>FR-DASH-15</t>
+        </is>
+      </c>
+      <c r="C72" s="2" t="inlineStr">
+        <is>
+          <t>ร้อยละของ 2 แถวคำนวณจากฐานที่ถูกต้องคนละฐาน</t>
+        </is>
+      </c>
+      <c r="D72" s="2" t="inlineStr">
+        <is>
+          <t>ค่าเริ่มต้น</t>
+        </is>
+      </c>
+      <c r="E72" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. เทียบร้อยละแถว 1 กับฐานเคสสะสมรวม
+2. เทียบร้อยละแถว 2 กับฐานรายใหม่วันนี้</t>
+        </is>
+      </c>
+      <c r="F72" s="2" t="inlineStr">
+        <is>
+          <t>แถวละฐานคนละฐานตามที่คำนวณจริง ไม่ใช้ฐานเดียวกัน</t>
+        </is>
+      </c>
+      <c r="G72" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H72" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I72" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J72" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="73" ht="60" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A73" s="2" t="inlineStr">
+        <is>
+          <t>TC-072</t>
+        </is>
+      </c>
+      <c r="B73" s="2" t="inlineStr">
+        <is>
+          <t>FR-DASH-15</t>
+        </is>
+      </c>
+      <c r="C73" s="2" t="inlineStr">
+        <is>
+          <t>ตารางป่วยจากอัปเดตตาม filter สอดคล้องกับ Stat Tiles</t>
+        </is>
+      </c>
+      <c r="D73" s="2" t="inlineStr">
+        <is>
+          <t>ค่าเริ่มต้น</t>
+        </is>
+      </c>
+      <c r="E73" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. เปลี่ยน filter ช่วงวันที่เป็น 7 วัน
+2. เทียบตารางป่วยจากกับ Stat Tiles ที่อัปเดตแล้ว</t>
+        </is>
+      </c>
+      <c r="F73" s="2" t="inlineStr">
+        <is>
+          <t>ตัวเลข 2 แถวเปลี่ยนตรงกับ Stat Tiles ที่คำนวณจาก filter เดียวกัน</t>
+        </is>
+      </c>
+      <c r="G73" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H73" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I73" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J73" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>